<commit_message>
Add validated sentiment evidence and unify the suite
</commit_message>
<xml_diff>
--- a/examples/textsignal-starter-template.xlsx
+++ b/examples/textsignal-starter-template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Text data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Text data'!$A$1:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Text data'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,12 +427,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,6 +453,31 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>recorded_at</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>human_sentiment</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>open_text</t>
         </is>
       </c>
@@ -463,7 +493,32 @@
           <t>Group A</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Brand A</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -476,7 +531,32 @@
           <t>Group B</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Brand A</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -489,7 +569,32 @@
           <t>Group A</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Brand B</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -502,10 +607,35 @@
           <t>Group B</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Brand B</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C5"/>
+  <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>